<commit_message>
refactor: centralize damage calculation with DamageCalculator
</commit_message>
<xml_diff>
--- a/Assets/DataSource/Excel/PlayerUpgrade.xlsx
+++ b/Assets/DataSource/Excel/PlayerUpgrade.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity_Project\Planet_Rogue\Assets\DataSource\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F1FDD39-ABAD-4D3A-BB34-66E97131C259}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DA76F96-D5BF-4D5B-B5AD-A70FD4293396}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,10 +69,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>critiDamageRate</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>maxJumpTimes</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -162,6 +158,10 @@
   </si>
   <si>
     <t>maxHpFlat</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>critiDamageMultiplier</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -490,13 +490,13 @@
   <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.625" customWidth="1"/>
+    <col min="1" max="1" width="21.75" customWidth="1"/>
     <col min="8" max="8" width="16.875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -522,7 +522,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B2">
         <v>10</v>
@@ -540,15 +540,15 @@
         <v>20</v>
       </c>
       <c r="G2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B3">
         <v>1.1000000000000001</v>
@@ -566,15 +566,15 @@
         <v>1.5</v>
       </c>
       <c r="G3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B4">
         <v>0.05</v>
@@ -592,10 +592,10 @@
         <v>0.3</v>
       </c>
       <c r="G4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -618,10 +618,10 @@
         <v>8</v>
       </c>
       <c r="G5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -644,10 +644,10 @@
         <v>7</v>
       </c>
       <c r="G6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
@@ -670,15 +670,15 @@
         <v>0.5</v>
       </c>
       <c r="G7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B8">
         <v>1.1000000000000001</v>
@@ -696,10 +696,10 @@
         <v>1.5</v>
       </c>
       <c r="G8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -722,10 +722,10 @@
         <v>1.8</v>
       </c>
       <c r="G9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -748,15 +748,15 @@
         <v>0.5</v>
       </c>
       <c r="G10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="B11">
         <v>2.1</v>
@@ -774,15 +774,15 @@
         <v>2.5</v>
       </c>
       <c r="G11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12">
         <v>2</v>
@@ -800,15 +800,15 @@
         <v>6</v>
       </c>
       <c r="G12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13">
         <v>7</v>
@@ -826,15 +826,15 @@
         <v>12</v>
       </c>
       <c r="G13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B14">
         <v>1.1000000000000001</v>
@@ -852,10 +852,10 @@
         <v>1.5</v>
       </c>
       <c r="G14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement player and weapon upgrade system
</commit_message>
<xml_diff>
--- a/Assets/DataSource/Excel/PlayerUpgrade.xlsx
+++ b/Assets/DataSource/Excel/PlayerUpgrade.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity_Project\Planet_Rogue\Assets\DataSource\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DA76F96-D5BF-4D5B-B5AD-A70FD4293396}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{300917F8-E276-4F5B-8CB7-B52A6EE41A28}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="37">
   <si>
     <t>armor</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -47,10 +47,6 @@
     <t>level5</t>
   </si>
   <si>
-    <t>type</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>description</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -129,22 +125,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>statsId</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>defRate</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>set</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>add</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>expRate</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -163,6 +147,25 @@
   <si>
     <t>critiDamageMultiplier</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>baseValue</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>stat</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Number</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>displayType</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Percent</t>
   </si>
 </sst>
 </file>
@@ -487,45 +490,49 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.75" customWidth="1"/>
+    <col min="2" max="2" width="12.75" customWidth="1"/>
     <col min="8" max="8" width="16.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B2">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C2">
         <v>10</v>
@@ -537,325 +544,364 @@
         <v>10</v>
       </c>
       <c r="F2">
+        <v>10</v>
+      </c>
+      <c r="G2">
         <v>20</v>
       </c>
-      <c r="G2" t="s">
-        <v>30</v>
-      </c>
       <c r="H2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+      <c r="I2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D3">
+        <v>1.2</v>
+      </c>
+      <c r="E3">
+        <v>1.3</v>
+      </c>
+      <c r="F3">
+        <v>1.4</v>
+      </c>
+      <c r="G3">
+        <v>1.5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>36</v>
+      </c>
+      <c r="I3" t="s">
         <v>14</v>
       </c>
-      <c r="B3">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="C3">
-        <v>1.2</v>
-      </c>
-      <c r="D3">
-        <v>1.3</v>
-      </c>
-      <c r="E3">
-        <v>1.4</v>
-      </c>
-      <c r="F3">
-        <v>1.5</v>
-      </c>
-      <c r="G3" t="s">
-        <v>29</v>
-      </c>
-      <c r="H3" t="s">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0.05</v>
+      </c>
+      <c r="D4">
+        <v>0.1</v>
+      </c>
+      <c r="E4">
+        <v>0.15</v>
+      </c>
+      <c r="F4">
+        <v>0.2</v>
+      </c>
+      <c r="G4">
+        <v>0.3</v>
+      </c>
+      <c r="H4" t="s">
+        <v>36</v>
+      </c>
+      <c r="I4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4">
-        <v>0.05</v>
-      </c>
-      <c r="C4">
-        <v>0.1</v>
-      </c>
-      <c r="D4">
-        <v>0.15</v>
-      </c>
-      <c r="E4">
-        <v>0.2</v>
-      </c>
-      <c r="F4">
-        <v>0.3</v>
-      </c>
-      <c r="G4" t="s">
-        <v>29</v>
-      </c>
-      <c r="H4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>0</v>
       </c>
       <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
         <v>1</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>2</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>3</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>5</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>8</v>
       </c>
-      <c r="G5" t="s">
-        <v>29</v>
-      </c>
       <c r="H5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6">
+        <v>4.5</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>5.5</v>
+      </c>
+      <c r="F6">
+        <v>6</v>
+      </c>
+      <c r="G6">
+        <v>7</v>
+      </c>
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>8</v>
       </c>
-      <c r="B6">
-        <v>4.5</v>
-      </c>
-      <c r="C6">
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>0.05</v>
+      </c>
+      <c r="D7">
+        <v>0.1</v>
+      </c>
+      <c r="E7">
+        <v>0.2</v>
+      </c>
+      <c r="F7">
+        <v>0.3</v>
+      </c>
+      <c r="G7">
+        <v>0.5</v>
+      </c>
+      <c r="H7" t="s">
+        <v>36</v>
+      </c>
+      <c r="I7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D8">
+        <v>1.2</v>
+      </c>
+      <c r="E8">
+        <v>1.3</v>
+      </c>
+      <c r="F8">
+        <v>1.4</v>
+      </c>
+      <c r="G8">
+        <v>1.5</v>
+      </c>
+      <c r="H8" t="s">
+        <v>36</v>
+      </c>
+      <c r="I8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1.2</v>
+      </c>
+      <c r="D9">
+        <v>1.3</v>
+      </c>
+      <c r="E9">
+        <v>1.4</v>
+      </c>
+      <c r="F9">
+        <v>1.5</v>
+      </c>
+      <c r="G9">
+        <v>1.8</v>
+      </c>
+      <c r="H9" t="s">
+        <v>36</v>
+      </c>
+      <c r="I9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>0.1</v>
+      </c>
+      <c r="D10">
+        <v>0.2</v>
+      </c>
+      <c r="E10">
+        <v>0.3</v>
+      </c>
+      <c r="F10">
+        <v>0.4</v>
+      </c>
+      <c r="G10">
+        <v>0.5</v>
+      </c>
+      <c r="H10" t="s">
+        <v>36</v>
+      </c>
+      <c r="I10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11">
+        <v>2.1</v>
+      </c>
+      <c r="D11">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="E11">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="F11">
+        <v>2.4</v>
+      </c>
+      <c r="G11">
+        <v>2.5</v>
+      </c>
+      <c r="H11" t="s">
+        <v>36</v>
+      </c>
+      <c r="I11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="E12">
+        <v>4</v>
+      </c>
+      <c r="F12">
         <v>5</v>
       </c>
-      <c r="D6">
-        <v>5.5</v>
-      </c>
-      <c r="E6">
+      <c r="G12">
         <v>6</v>
       </c>
-      <c r="F6">
+      <c r="H12" t="s">
+        <v>34</v>
+      </c>
+      <c r="I12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>6</v>
+      </c>
+      <c r="C13">
         <v>7</v>
       </c>
-      <c r="G6" t="s">
-        <v>29</v>
-      </c>
-      <c r="H6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="D13">
+        <v>8</v>
+      </c>
+      <c r="E13">
         <v>9</v>
       </c>
-      <c r="B7">
-        <v>0.05</v>
-      </c>
-      <c r="C7">
-        <v>0.1</v>
-      </c>
-      <c r="D7">
-        <v>0.2</v>
-      </c>
-      <c r="E7">
-        <v>0.3</v>
-      </c>
-      <c r="F7">
-        <v>0.5</v>
-      </c>
-      <c r="G7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8">
+      <c r="F13">
+        <v>10</v>
+      </c>
+      <c r="G13">
+        <v>12</v>
+      </c>
+      <c r="H13" t="s">
+        <v>34</v>
+      </c>
+      <c r="I13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14">
         <v>1.1000000000000001</v>
       </c>
-      <c r="C8">
+      <c r="D14">
         <v>1.2</v>
       </c>
-      <c r="D8">
+      <c r="E14">
         <v>1.3</v>
       </c>
-      <c r="E8">
+      <c r="F14">
         <v>1.4</v>
       </c>
-      <c r="F8">
+      <c r="G14">
         <v>1.5</v>
       </c>
-      <c r="G8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9">
-        <v>1.2</v>
-      </c>
-      <c r="C9">
-        <v>1.3</v>
-      </c>
-      <c r="D9">
-        <v>1.4</v>
-      </c>
-      <c r="E9">
-        <v>1.5</v>
-      </c>
-      <c r="F9">
-        <v>1.8</v>
-      </c>
-      <c r="G9" t="s">
-        <v>29</v>
-      </c>
-      <c r="H9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10">
-        <v>0.1</v>
-      </c>
-      <c r="C10">
-        <v>0.2</v>
-      </c>
-      <c r="D10">
-        <v>0.3</v>
-      </c>
-      <c r="E10">
-        <v>0.4</v>
-      </c>
-      <c r="F10">
-        <v>0.5</v>
-      </c>
-      <c r="G10" t="s">
-        <v>29</v>
-      </c>
-      <c r="H10" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>35</v>
-      </c>
-      <c r="B11">
-        <v>2.1</v>
-      </c>
-      <c r="C11">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="D11">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="E11">
-        <v>2.4</v>
-      </c>
-      <c r="F11">
-        <v>2.5</v>
-      </c>
-      <c r="G11" t="s">
-        <v>29</v>
-      </c>
-      <c r="H11" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12">
-        <v>2</v>
-      </c>
-      <c r="C12">
-        <v>3</v>
-      </c>
-      <c r="D12">
-        <v>4</v>
-      </c>
-      <c r="E12">
-        <v>5</v>
-      </c>
-      <c r="F12">
-        <v>6</v>
-      </c>
-      <c r="G12" t="s">
-        <v>29</v>
-      </c>
-      <c r="H12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13">
-        <v>7</v>
-      </c>
-      <c r="C13">
-        <v>8</v>
-      </c>
-      <c r="D13">
-        <v>9</v>
-      </c>
-      <c r="E13">
-        <v>10</v>
-      </c>
-      <c r="F13">
-        <v>12</v>
-      </c>
-      <c r="G13" t="s">
-        <v>29</v>
-      </c>
-      <c r="H13" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>31</v>
-      </c>
-      <c r="B14">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="C14">
-        <v>1.2</v>
-      </c>
-      <c r="D14">
-        <v>1.3</v>
-      </c>
-      <c r="E14">
-        <v>1.4</v>
-      </c>
-      <c r="F14">
-        <v>1.5</v>
-      </c>
-      <c r="G14" t="s">
-        <v>29</v>
-      </c>
       <c r="H14" t="s">
-        <v>32</v>
+        <v>36</v>
+      </c>
+      <c r="I14" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
balance: adjust player movement and jump values
</commit_message>
<xml_diff>
--- a/Assets/DataSource/Excel/PlayerUpgrade.xlsx
+++ b/Assets/DataSource/Excel/PlayerUpgrade.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity_Project\Planet_Rogue\Assets\DataSource\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{300917F8-E276-4F5B-8CB7-B52A6EE41A28}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E5888B4-E700-41E6-B209-5491CACA3D0E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -648,22 +648,22 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C6">
-        <v>4.5</v>
+        <v>6.5</v>
       </c>
       <c r="D6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E6">
-        <v>5.5</v>
+        <v>7.5</v>
       </c>
       <c r="F6">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G6">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H6" t="s">
         <v>34</v>
@@ -851,22 +851,22 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C13">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D13">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E13">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F13">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G13">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="H13" t="s">
         <v>34</v>

</xml_diff>

<commit_message>
fix: initialize player stats from config data
- Apply base stat values from PlayerUpgrade.json on initialization
- Replace hardcoded player stat defaults with config values
- Simplify max HP handling and remove maxHpFlat
- Rename MaxHpFlat stat to MaxHp
</commit_message>
<xml_diff>
--- a/Assets/DataSource/Excel/PlayerUpgrade.xlsx
+++ b/Assets/DataSource/Excel/PlayerUpgrade.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity_Project\Planet_Rogue\Assets\DataSource\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E5888B4-E700-41E6-B209-5491CACA3D0E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E1CCB38-D454-4988-A4A9-C5AD6D42ABCF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -141,10 +141,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>maxHpFlat</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>critiDamageMultiplier</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -166,6 +162,10 @@
   </si>
   <si>
     <t>Percent</t>
+  </si>
+  <si>
+    <t>maxHp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -500,10 +500,10 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -521,7 +521,7 @@
         <v>5</v>
       </c>
       <c r="H1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I1" t="s">
         <v>6</v>
@@ -529,28 +529,28 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C2">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="D2">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="E2">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="F2">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="G2">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="H2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I2" t="s">
         <v>29</v>
@@ -579,7 +579,7 @@
         <v>1.5</v>
       </c>
       <c r="H3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I3" t="s">
         <v>14</v>
@@ -608,7 +608,7 @@
         <v>0.3</v>
       </c>
       <c r="H4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I4" t="s">
         <v>15</v>
@@ -637,7 +637,7 @@
         <v>8</v>
       </c>
       <c r="H5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I5" t="s">
         <v>16</v>
@@ -648,16 +648,16 @@
         <v>7</v>
       </c>
       <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6">
         <v>6</v>
       </c>
-      <c r="C6">
-        <v>6.5</v>
-      </c>
-      <c r="D6">
+      <c r="E6">
         <v>7</v>
-      </c>
-      <c r="E6">
-        <v>7.5</v>
       </c>
       <c r="F6">
         <v>8</v>
@@ -666,7 +666,7 @@
         <v>9</v>
       </c>
       <c r="H6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I6" t="s">
         <v>17</v>
@@ -695,7 +695,7 @@
         <v>0.5</v>
       </c>
       <c r="H7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I7" t="s">
         <v>18</v>
@@ -724,7 +724,7 @@
         <v>1.5</v>
       </c>
       <c r="H8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I8" t="s">
         <v>19</v>
@@ -753,7 +753,7 @@
         <v>1.8</v>
       </c>
       <c r="H9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I9" t="s">
         <v>20</v>
@@ -782,7 +782,7 @@
         <v>0.5</v>
       </c>
       <c r="H10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I10" t="s">
         <v>21</v>
@@ -790,7 +790,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B11">
         <v>2</v>
@@ -811,7 +811,7 @@
         <v>2.5</v>
       </c>
       <c r="H11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I11" t="s">
         <v>22</v>
@@ -840,7 +840,7 @@
         <v>6</v>
       </c>
       <c r="H12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I12" t="s">
         <v>23</v>
@@ -851,25 +851,25 @@
         <v>12</v>
       </c>
       <c r="B13">
+        <v>6</v>
+      </c>
+      <c r="C13">
+        <v>7</v>
+      </c>
+      <c r="D13">
+        <v>8</v>
+      </c>
+      <c r="E13">
+        <v>9</v>
+      </c>
+      <c r="F13">
         <v>10</v>
       </c>
-      <c r="C13">
-        <v>11</v>
-      </c>
-      <c r="D13">
+      <c r="G13">
         <v>12</v>
       </c>
-      <c r="E13">
-        <v>13</v>
-      </c>
-      <c r="F13">
-        <v>14</v>
-      </c>
-      <c r="G13">
-        <v>16</v>
-      </c>
       <c r="H13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I13" t="s">
         <v>24</v>
@@ -898,7 +898,7 @@
         <v>1.5</v>
       </c>
       <c r="H14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I14" t="s">
         <v>28</v>

</xml_diff>